<commit_message>
fix(demo): UPG-1 Spool Revision is the ISO revision, as in the manual
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/demo-project/UPG-1.xlsx
+++ b/fixtures/demo-project/UPG-1.xlsx
@@ -4675,8 +4675,8 @@
       <c r="P2" t="str">
         <v>UPG-100-1001-S1</v>
       </c>
-      <c r="Q2">
-        <v>1</v>
+      <c r="Q2" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="3">
@@ -4728,8 +4728,8 @@
       <c r="P3" t="str">
         <v>UPG-100-1002-S1</v>
       </c>
-      <c r="Q3">
-        <v>1</v>
+      <c r="Q3" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="4">
@@ -4781,8 +4781,8 @@
       <c r="P4" t="str">
         <v>UPG-100-1003-S1</v>
       </c>
-      <c r="Q4">
-        <v>1</v>
+      <c r="Q4" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="5">
@@ -4834,8 +4834,8 @@
       <c r="P5" t="str">
         <v>UPG-100-1004-S1</v>
       </c>
-      <c r="Q5">
-        <v>1</v>
+      <c r="Q5" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="6">
@@ -4887,8 +4887,8 @@
       <c r="P6" t="str">
         <v>UPG-100-1005-S1</v>
       </c>
-      <c r="Q6">
-        <v>1</v>
+      <c r="Q6" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="7">
@@ -4940,8 +4940,8 @@
       <c r="P7" t="str">
         <v>UPG-100-1006-S1</v>
       </c>
-      <c r="Q7">
-        <v>1</v>
+      <c r="Q7" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="8">
@@ -4993,8 +4993,8 @@
       <c r="P8" t="str">
         <v>UPG-100-1007-S1</v>
       </c>
-      <c r="Q8">
-        <v>1</v>
+      <c r="Q8" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="9">
@@ -5046,8 +5046,8 @@
       <c r="P9" t="str">
         <v>UPG-100-1008-S1</v>
       </c>
-      <c r="Q9">
-        <v>1</v>
+      <c r="Q9" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="10">
@@ -5099,8 +5099,8 @@
       <c r="P10" t="str">
         <v>UPG-100-1009-S1</v>
       </c>
-      <c r="Q10">
-        <v>1</v>
+      <c r="Q10" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="11">
@@ -5152,8 +5152,8 @@
       <c r="P11" t="str">
         <v>UPG-100-1010-S1</v>
       </c>
-      <c r="Q11">
-        <v>1</v>
+      <c r="Q11" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="12">
@@ -5205,8 +5205,8 @@
       <c r="P12" t="str">
         <v>UPG-200-2001-S1</v>
       </c>
-      <c r="Q12">
-        <v>1</v>
+      <c r="Q12" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="13">
@@ -5258,8 +5258,8 @@
       <c r="P13" t="str">
         <v>UPG-200-2002-S1</v>
       </c>
-      <c r="Q13">
-        <v>1</v>
+      <c r="Q13" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="14">
@@ -5311,8 +5311,8 @@
       <c r="P14" t="str">
         <v>UPG-200-2003-S1</v>
       </c>
-      <c r="Q14">
-        <v>1</v>
+      <c r="Q14" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="15">
@@ -5364,8 +5364,8 @@
       <c r="P15" t="str">
         <v>UPG-200-2004-S1</v>
       </c>
-      <c r="Q15">
-        <v>1</v>
+      <c r="Q15" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="16">
@@ -5417,8 +5417,8 @@
       <c r="P16" t="str">
         <v>UPG-200-2005-S1</v>
       </c>
-      <c r="Q16">
-        <v>1</v>
+      <c r="Q16" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="17">
@@ -5470,8 +5470,8 @@
       <c r="P17" t="str">
         <v>UPG-200-2006-S1</v>
       </c>
-      <c r="Q17">
-        <v>1</v>
+      <c r="Q17" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="18">
@@ -5523,8 +5523,8 @@
       <c r="P18" t="str">
         <v>UPG-200-2007-S1</v>
       </c>
-      <c r="Q18">
-        <v>1</v>
+      <c r="Q18" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="19">
@@ -5576,8 +5576,8 @@
       <c r="P19" t="str">
         <v>UPG-200-2008-S1</v>
       </c>
-      <c r="Q19">
-        <v>1</v>
+      <c r="Q19" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="20">
@@ -5629,8 +5629,8 @@
       <c r="P20" t="str">
         <v>UPG-200-2009-S1</v>
       </c>
-      <c r="Q20">
-        <v>1</v>
+      <c r="Q20" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="21">
@@ -5682,8 +5682,8 @@
       <c r="P21" t="str">
         <v>UPG-200-2010-S1</v>
       </c>
-      <c r="Q21">
-        <v>1</v>
+      <c r="Q21" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="22">
@@ -5735,8 +5735,8 @@
       <c r="P22" t="str">
         <v>UPG-200-2011-S1</v>
       </c>
-      <c r="Q22">
-        <v>1</v>
+      <c r="Q22" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="23">
@@ -5788,8 +5788,8 @@
       <c r="P23" t="str">
         <v>UPG-200-2012-S1</v>
       </c>
-      <c r="Q23">
-        <v>1</v>
+      <c r="Q23" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="24">
@@ -5841,8 +5841,8 @@
       <c r="P24" t="str">
         <v>UPG-300-3001-S1</v>
       </c>
-      <c r="Q24">
-        <v>1</v>
+      <c r="Q24" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="25">
@@ -5894,8 +5894,8 @@
       <c r="P25" t="str">
         <v>UPG-300-3002-S1</v>
       </c>
-      <c r="Q25">
-        <v>1</v>
+      <c r="Q25" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="26">
@@ -5947,8 +5947,8 @@
       <c r="P26" t="str">
         <v>UPG-300-3003-S1</v>
       </c>
-      <c r="Q26">
-        <v>1</v>
+      <c r="Q26" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="27">
@@ -6000,8 +6000,8 @@
       <c r="P27" t="str">
         <v>UPG-300-3004-S1</v>
       </c>
-      <c r="Q27">
-        <v>1</v>
+      <c r="Q27" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="28">
@@ -6053,8 +6053,8 @@
       <c r="P28" t="str">
         <v>UPG-300-3005-S1</v>
       </c>
-      <c r="Q28">
-        <v>1</v>
+      <c r="Q28" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="29">
@@ -6106,8 +6106,8 @@
       <c r="P29" t="str">
         <v>UPG-300-3006-S1</v>
       </c>
-      <c r="Q29">
-        <v>1</v>
+      <c r="Q29" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="30">
@@ -6159,8 +6159,8 @@
       <c r="P30" t="str">
         <v>UPG-300-3007-S1</v>
       </c>
-      <c r="Q30">
-        <v>1</v>
+      <c r="Q30" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="31">
@@ -6212,8 +6212,8 @@
       <c r="P31" t="str">
         <v>UPG-300-3008-S1</v>
       </c>
-      <c r="Q31">
-        <v>1</v>
+      <c r="Q31" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="32">
@@ -6265,8 +6265,8 @@
       <c r="P32" t="str">
         <v>UPG-300-3009-S1</v>
       </c>
-      <c r="Q32">
-        <v>1</v>
+      <c r="Q32" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="33">
@@ -6318,8 +6318,8 @@
       <c r="P33" t="str">
         <v>UPG-300-3010-S1</v>
       </c>
-      <c r="Q33">
-        <v>1</v>
+      <c r="Q33" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="34">
@@ -6371,8 +6371,8 @@
       <c r="P34" t="str">
         <v>UPG-300-3011-S1</v>
       </c>
-      <c r="Q34">
-        <v>1</v>
+      <c r="Q34" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="35">
@@ -6424,8 +6424,8 @@
       <c r="P35" t="str">
         <v>UPG-300-3012-S1</v>
       </c>
-      <c r="Q35">
-        <v>1</v>
+      <c r="Q35" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="36">
@@ -6477,8 +6477,8 @@
       <c r="P36" t="str">
         <v>UPG-300-3013-S1</v>
       </c>
-      <c r="Q36">
-        <v>1</v>
+      <c r="Q36" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="37">
@@ -6530,8 +6530,8 @@
       <c r="P37" t="str">
         <v>UPG-300-3014-S1</v>
       </c>
-      <c r="Q37">
-        <v>1</v>
+      <c r="Q37" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="38">
@@ -6583,8 +6583,8 @@
       <c r="P38" t="str">
         <v>UPG-300-3015-S1</v>
       </c>
-      <c r="Q38">
-        <v>1</v>
+      <c r="Q38" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="39">
@@ -6636,8 +6636,8 @@
       <c r="P39" t="str">
         <v>UPG-300-3016-S1</v>
       </c>
-      <c r="Q39">
-        <v>1</v>
+      <c r="Q39" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="40">
@@ -6689,8 +6689,8 @@
       <c r="P40" t="str">
         <v>UPG-300-3017-S1</v>
       </c>
-      <c r="Q40">
-        <v>1</v>
+      <c r="Q40" t="str">
+        <v>R0</v>
       </c>
     </row>
     <row r="41">
@@ -6742,8 +6742,8 @@
       <c r="P41" t="str">
         <v>UPG-300-3018-S1</v>
       </c>
-      <c r="Q41">
-        <v>1</v>
+      <c r="Q41" t="str">
+        <v>R0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(import): WPS and welder dates come from the file, not from the server clock
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/demo-project/UPG-1.xlsx
+++ b/fixtures/demo-project/UPG-1.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,27 +437,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>5. В терминале: npm run demo:project-setup -- --project UPG-1 --phase backdate-wps</v>
+        <v>5. Спулинг → Импорт: сначала error/weld.txt (ожидаем блокер), затем spooling/weld, trace, bolt, supp.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6. Спулинг → Импорт: сначала error/weld.txt (ожидаем блокер), затем spooling/weld, trace, bolt, supp.</v>
+        <v>6. Test Packs → Импорт состава: imports/06-test-packs.xlsx.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>7. Test Packs → Импорт состава: imports/06-test-packs.xlsx.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>8. Неделя 3: Спулинг → Импорт revision/*.txt и решения по ревизии.</v>
+        <v>7. Неделя 3: Спулинг → Импорт revision/*.txt и решения по ревизии.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7327,7 +7322,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7351,6 +7346,9 @@
       <c r="G1" t="str">
         <v>Thickness To</v>
       </c>
+      <c r="H1" t="str">
+        <v>Approved On</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7374,6 +7372,9 @@
       <c r="G2">
         <v>40</v>
       </c>
+      <c r="H2" t="str">
+        <v>2026-07-31</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7397,6 +7398,9 @@
       <c r="G3">
         <v>20</v>
       </c>
+      <c r="H3" t="str">
+        <v>2026-07-31</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -7420,6 +7424,9 @@
       <c r="G4">
         <v>40</v>
       </c>
+      <c r="H4" t="str">
+        <v>2026-07-31</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -7443,17 +7450,20 @@
       <c r="G5">
         <v>20</v>
       </c>
+      <c r="H5" t="str">
+        <v>2026-07-31</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7468,6 +7478,9 @@
       <c r="D1" t="str">
         <v>WPS Codes</v>
       </c>
+      <c r="E1" t="str">
+        <v>Expires On</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7482,6 +7495,9 @@
       <c r="D2" t="str">
         <v>WPS-CS-01,WPS-SS-01</v>
       </c>
+      <c r="E2" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7496,6 +7512,9 @@
       <c r="D3" t="str">
         <v>WPS-CS-01,WPS-SS-01</v>
       </c>
+      <c r="E3" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -7510,6 +7529,9 @@
       <c r="D4" t="str">
         <v>WPS-CS-01</v>
       </c>
+      <c r="E4" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -7524,6 +7546,9 @@
       <c r="D5" t="str">
         <v>WPS-CS-01</v>
       </c>
+      <c r="E5" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -7538,6 +7563,9 @@
       <c r="D6" t="str">
         <v>WPS-CS-01,WPS-SS-01</v>
       </c>
+      <c r="E6" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -7552,6 +7580,9 @@
       <c r="D7" t="str">
         <v>WPS-SS-01</v>
       </c>
+      <c r="E7" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -7566,6 +7597,9 @@
       <c r="D8" t="str">
         <v>WPS-CS-F01,WPS-SS-F01</v>
       </c>
+      <c r="E8" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -7580,6 +7614,9 @@
       <c r="D9" t="str">
         <v>WPS-CS-F01</v>
       </c>
+      <c r="E9" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -7594,6 +7631,9 @@
       <c r="D10" t="str">
         <v>WPS-CS-F01,WPS-SS-F01</v>
       </c>
+      <c r="E10" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -7608,10 +7648,13 @@
       <c r="D11" t="str">
         <v>WPS-SS-F01</v>
       </c>
+      <c r="E11" t="str">
+        <v>2028-08-13</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>